<commit_message>
Update Script to have section C
</commit_message>
<xml_diff>
--- a/Q4_Results.xlsx
+++ b/Q4_Results.xlsx
@@ -8,13 +8,14 @@
   <sheets>
     <sheet name="Angular Velocities" sheetId="1" r:id="rId2"/>
     <sheet name="Angular Accelerations" sheetId="2" r:id="rId4"/>
+    <sheet name="Pin A" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="70" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="91" uniqueCount="19">
   <si>
     <t>Theta2_deg</t>
   </si>
@@ -53,6 +54,24 @@
   </si>
   <si>
     <t>alpha8</t>
+  </si>
+  <si>
+    <t>X_A_mm</t>
+  </si>
+  <si>
+    <t>Y_A_mm</t>
+  </si>
+  <si>
+    <t>Vx_A_mm_s</t>
+  </si>
+  <si>
+    <t>Vy_A_mm_s</t>
+  </si>
+  <si>
+    <t>Ax_A_mm_s2</t>
+  </si>
+  <si>
+    <t>Ay_A_mm_s2</t>
   </si>
 </sst>
 </file>
@@ -5742,4 +5761,2828 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G122"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" customWidth="true"/>
+    <col min="2" max="2" width="12.42578125" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="12.42578125" customWidth="true"/>
+    <col min="5" max="5" width="12.42578125" customWidth="true"/>
+    <col min="6" max="6" width="13" customWidth="true"/>
+    <col min="7" max="7" width="13" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0">
+        <v>0</v>
+      </c>
+      <c r="B2" s="0">
+        <v>-471.49874012952415</v>
+      </c>
+      <c r="C2" s="0">
+        <v>237.11108660256895</v>
+      </c>
+      <c r="D2" s="0">
+        <v>-1.8860645306442123</v>
+      </c>
+      <c r="E2" s="0">
+        <v>1171.2908885536772</v>
+      </c>
+      <c r="F2" s="0">
+        <v>-1944.3500311672851</v>
+      </c>
+      <c r="G2" s="0">
+        <v>-10919.399512360818</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>1</v>
+      </c>
+      <c r="B3" s="0">
+        <v>-471.79612246133712</v>
+      </c>
+      <c r="C3" s="0">
+        <v>256.19038243929629</v>
+      </c>
+      <c r="D3" s="0">
+        <v>-30.727452697519148</v>
+      </c>
+      <c r="E3" s="0">
+        <v>1028.6877247023658</v>
+      </c>
+      <c r="F3" s="0">
+        <v>-1432.4541829766843</v>
+      </c>
+      <c r="G3" s="0">
+        <v>-6137.2795643993741</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>2</v>
+      </c>
+      <c r="B4" s="0">
+        <v>-472.53618144016076</v>
+      </c>
+      <c r="C4" s="0">
+        <v>273.33842146836969</v>
+      </c>
+      <c r="D4" s="0">
+        <v>-53.371952557588379</v>
+      </c>
+      <c r="E4" s="0">
+        <v>942.55631268094044</v>
+      </c>
+      <c r="F4" s="0">
+        <v>-1187.8348328610837</v>
+      </c>
+      <c r="G4" s="0">
+        <v>-3975.5972085434319</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>3</v>
+      </c>
+      <c r="B5" s="0">
+        <v>-473.64064073144931</v>
+      </c>
+      <c r="C5" s="0">
+        <v>289.25134996277547</v>
+      </c>
+      <c r="D5" s="0">
+        <v>-72.786668705656027</v>
+      </c>
+      <c r="E5" s="0">
+        <v>884.31427143568294</v>
+      </c>
+      <c r="F5" s="0">
+        <v>-1048.4581410131295</v>
+      </c>
+      <c r="G5" s="0">
+        <v>-2804.7345621523145</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>4</v>
+      </c>
+      <c r="B6" s="0">
+        <v>-475.06573986573477</v>
+      </c>
+      <c r="C6" s="0">
+        <v>304.29846255927316</v>
+      </c>
+      <c r="D6" s="0">
+        <v>-90.261671764151259</v>
+      </c>
+      <c r="E6" s="0">
+        <v>842.00428715974613</v>
+      </c>
+      <c r="F6" s="0">
+        <v>-960.10164411683002</v>
+      </c>
+      <c r="G6" s="0">
+        <v>-2097.9007833810706</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>5</v>
+      </c>
+      <c r="B7" s="0">
+        <v>-476.7840029012167</v>
+      </c>
+      <c r="C7" s="0">
+        <v>318.70034198519755</v>
+      </c>
+      <c r="D7" s="0">
+        <v>-106.46202607868307</v>
+      </c>
+      <c r="E7" s="0">
+        <v>809.65856961734346</v>
+      </c>
+      <c r="F7" s="0">
+        <v>-899.85276444385841</v>
+      </c>
+      <c r="G7" s="0">
+        <v>-1639.3981824817647</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>6</v>
+      </c>
+      <c r="B8" s="0">
+        <v>-478.77679926375004</v>
+      </c>
+      <c r="C8" s="0">
+        <v>332.59919130717782</v>
+      </c>
+      <c r="D8" s="0">
+        <v>-121.7697456629698</v>
+      </c>
+      <c r="E8" s="0">
+        <v>783.9397844129835</v>
+      </c>
+      <c r="F8" s="0">
+        <v>-856.48433445154717</v>
+      </c>
+      <c r="G8" s="0">
+        <v>-1326.5433304116023</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>7</v>
+      </c>
+      <c r="B9" s="0">
+        <v>-481.03076638291765</v>
+      </c>
+      <c r="C9" s="0">
+        <v>346.09166150615647</v>
+      </c>
+      <c r="D9" s="0">
+        <v>-136.4212406288022</v>
+      </c>
+      <c r="E9" s="0">
+        <v>762.82632885085593</v>
+      </c>
+      <c r="F9" s="0">
+        <v>-823.89881335487394</v>
+      </c>
+      <c r="G9" s="0">
+        <v>-1105.0249083316696</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>8</v>
+      </c>
+      <c r="B10" s="0">
+        <v>-483.53588883557501</v>
+      </c>
+      <c r="C10" s="0">
+        <v>359.24600639311956</v>
+      </c>
+      <c r="D10" s="0">
+        <v>-150.57093883098568</v>
+      </c>
+      <c r="E10" s="0">
+        <v>745.018698018583</v>
+      </c>
+      <c r="F10" s="0">
+        <v>-798.5238946374111</v>
+      </c>
+      <c r="G10" s="0">
+        <v>-943.78537960574647</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>9</v>
+      </c>
+      <c r="B11" s="0">
+        <v>-486.28438136315413</v>
+      </c>
+      <c r="C11" s="0">
+        <v>372.11181479801206</v>
+      </c>
+      <c r="D11" s="0">
+        <v>-164.32388317025874</v>
+      </c>
+      <c r="E11" s="0">
+        <v>729.64232841387059</v>
+      </c>
+      <c r="F11" s="0">
+        <v>-778.14146151504099</v>
+      </c>
+      <c r="G11" s="0">
+        <v>-823.96197913835965</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>10</v>
+      </c>
+      <c r="B12" s="0">
+        <v>-489.26999888625306</v>
+      </c>
+      <c r="C12" s="0">
+        <v>384.72588876149666</v>
+      </c>
+      <c r="D12" s="0">
+        <v>-177.7537674959606</v>
+      </c>
+      <c r="E12" s="0">
+        <v>716.08673392960589</v>
+      </c>
+      <c r="F12" s="0">
+        <v>-761.30947321502674</v>
+      </c>
+      <c r="G12" s="0">
+        <v>-733.53562099454246</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>11</v>
+      </c>
+      <c r="B13" s="0">
+        <v>-492.48758959841177</v>
+      </c>
+      <c r="C13" s="0">
+        <v>397.11597401403009</v>
+      </c>
+      <c r="D13" s="0">
+        <v>-190.91353594667612</v>
+      </c>
+      <c r="E13" s="0">
+        <v>703.91288471494374</v>
+      </c>
+      <c r="F13" s="0">
+        <v>-747.05489783205076</v>
+      </c>
+      <c r="G13" s="0">
+        <v>-664.54249417936444</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0">
+        <v>12</v>
+      </c>
+      <c r="B14" s="0">
+        <v>-495.93279424685977</v>
+      </c>
+      <c r="C14" s="0">
+        <v>409.30322434448425</v>
+      </c>
+      <c r="D14" s="0">
+        <v>-203.84192212086595</v>
+      </c>
+      <c r="E14" s="0">
+        <v>692.79715062334651</v>
+      </c>
+      <c r="F14" s="0">
+        <v>-734.7007100486461</v>
+      </c>
+      <c r="G14" s="0">
+        <v>-611.53143486433862</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0">
+        <v>13</v>
+      </c>
+      <c r="B15" s="0">
+        <v>-499.60183733904842</v>
+      </c>
+      <c r="C15" s="0">
+        <v>421.30388453220644</v>
+      </c>
+      <c r="D15" s="0">
+        <v>-216.5676480060051</v>
+      </c>
+      <c r="E15" s="0">
+        <v>682.49594644388378</v>
+      </c>
+      <c r="F15" s="0">
+        <v>-723.76357567147181</v>
+      </c>
+      <c r="G15" s="0">
+        <v>-570.66727968981002</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0">
+        <v>14</v>
+      </c>
+      <c r="B16" s="0">
+        <v>-503.49137833071399</v>
+      </c>
+      <c r="C16" s="0">
+        <v>433.13047221334222</v>
+      </c>
+      <c r="D16" s="0">
+        <v>-229.11221205215966</v>
+      </c>
+      <c r="E16" s="0">
+        <v>672.82264722094965</v>
+      </c>
+      <c r="F16" s="0">
+        <v>-713.89083150783836</v>
+      </c>
+      <c r="G16" s="0">
+        <v>-539.18760915552798</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0">
+        <v>15</v>
+      </c>
+      <c r="B17" s="0">
+        <v>-507.59840318954071</v>
+      </c>
+      <c r="C17" s="0">
+        <v>444.79262791883389</v>
+      </c>
+      <c r="D17" s="0">
+        <v>-241.49179390003204</v>
+      </c>
+      <c r="E17" s="0">
+        <v>663.63206303041295</v>
+      </c>
+      <c r="F17" s="0">
+        <v>-704.8203051438802</v>
+      </c>
+      <c r="G17" s="0">
+        <v>-515.06175127824167</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0">
+        <v>16</v>
+      </c>
+      <c r="B18" s="0">
+        <v>-511.92014386929981</v>
+      </c>
+      <c r="C18" s="0">
+        <v>456.29773919776335</v>
+      </c>
+      <c r="D18" s="0">
+        <v>-253.71858789293287</v>
+      </c>
+      <c r="E18" s="0">
+        <v>654.8097279250162</v>
+      </c>
+      <c r="F18" s="0">
+        <v>-696.35392488447746</v>
+      </c>
+      <c r="G18" s="0">
+        <v>-496.77011041978818</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0">
+        <v>17</v>
+      </c>
+      <c r="B19" s="0">
+        <v>-516.45401752604994</v>
+      </c>
+      <c r="C19" s="0">
+        <v>467.65140720219517</v>
+      </c>
+      <c r="D19" s="0">
+        <v>-265.80175676923977</v>
+      </c>
+      <c r="E19" s="0">
+        <v>646.26434398770198</v>
+      </c>
+      <c r="F19" s="0">
+        <v>-688.33993399783333</v>
+      </c>
+      <c r="G19" s="0">
+        <v>-483.15751430900451</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0">
+        <v>18</v>
+      </c>
+      <c r="B20" s="0">
+        <v>-521.19757998147122</v>
+      </c>
+      <c r="C20" s="0">
+        <v>478.857801085201</v>
+      </c>
+      <c r="D20" s="0">
+        <v>-277.74812658642702</v>
+      </c>
+      <c r="E20" s="0">
+        <v>637.92234573402425</v>
+      </c>
+      <c r="F20" s="0">
+        <v>-680.66062969872712</v>
+      </c>
+      <c r="G20" s="0">
+        <v>-473.3334458353217</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0">
+        <v>19</v>
+      </c>
+      <c r="B21" s="0">
+        <v>-526.14848965112037</v>
+      </c>
+      <c r="C21" s="0">
+        <v>489.91993101429711</v>
+      </c>
+      <c r="D21" s="0">
+        <v>-289.56270153819571</v>
+      </c>
+      <c r="E21" s="0">
+        <v>629.72392136789381</v>
+      </c>
+      <c r="F21" s="0">
+        <v>-673.22374011861052</v>
+      </c>
+      <c r="G21" s="0">
+        <v>-466.60274936930642</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0">
+        <v>20</v>
+      </c>
+      <c r="B22" s="0">
+        <v>-531.30447928105502</v>
+      </c>
+      <c r="C22" s="0">
+        <v>500.83986116443748</v>
+      </c>
+      <c r="D22" s="0">
+        <v>-301.24905101663666</v>
+      </c>
+      <c r="E22" s="0">
+        <v>621.62005490440731</v>
+      </c>
+      <c r="F22" s="0">
+        <v>-665.95625101495341</v>
+      </c>
+      <c r="G22" s="0">
+        <v>-462.41660485881619</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0">
+        <v>21</v>
+      </c>
+      <c r="B23" s="0">
+        <v>-536.66333359305963</v>
+      </c>
+      <c r="C23" s="0">
+        <v>511.61887778812388</v>
+      </c>
+      <c r="D23" s="0">
+        <v>-312.80960450919133</v>
+      </c>
+      <c r="E23" s="0">
+        <v>613.57029635095239</v>
+      </c>
+      <c r="F23" s="0">
+        <v>-658.79991531838004</v>
+      </c>
+      <c r="G23" s="0">
+        <v>-460.33726099668752</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0">
+        <v>22</v>
+      </c>
+      <c r="B24" s="0">
+        <v>-542.22287145788721</v>
+      </c>
+      <c r="C24" s="0">
+        <v>522.25762321229604</v>
+      </c>
+      <c r="D24" s="0">
+        <v>-324.24587898894401</v>
+      </c>
+      <c r="E24" s="0">
+        <v>605.54105940945794</v>
+      </c>
+      <c r="F24" s="0">
+        <v>-651.7079395834802</v>
+      </c>
+      <c r="G24" s="0">
+        <v>-460.01228306338345</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0">
+        <v>23</v>
+      </c>
+      <c r="B25" s="0">
+        <v>-547.98093157856761</v>
+      </c>
+      <c r="C25" s="0">
+        <v>532.75620367757597</v>
+      </c>
+      <c r="D25" s="0">
+        <v>-335.55865617737175</v>
+      </c>
+      <c r="E25" s="0">
+        <v>597.50430691211261</v>
+      </c>
+      <c r="F25" s="0">
+        <v>-644.64250692164171</v>
+      </c>
+      <c r="G25" s="0">
+        <v>-461.15549123338821</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0">
+        <v>24</v>
+      </c>
+      <c r="B26" s="0">
+        <v>-553.93536092336444</v>
+      </c>
+      <c r="C26" s="0">
+        <v>543.11427687461139</v>
+      </c>
+      <c r="D26" s="0">
+        <v>-346.74812211895659</v>
+      </c>
+      <c r="E26" s="0">
+        <v>589.43652497745632</v>
+      </c>
+      <c r="F26" s="0">
+        <v>-637.57290323563245</v>
+      </c>
+      <c r="G26" s="0">
+        <v>-463.53267544933749</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0">
+        <v>25</v>
+      </c>
+      <c r="B27" s="0">
+        <v>-560.08400533349618</v>
+      </c>
+      <c r="C27" s="0">
+        <v>553.33112356223285</v>
+      </c>
+      <c r="D27" s="0">
+        <v>-357.81397809715327</v>
+      </c>
+      <c r="E27" s="0">
+        <v>581.31791472574435</v>
+      </c>
+      <c r="F27" s="0">
+        <v>-630.47408442175163</v>
+      </c>
+      <c r="G27" s="0">
+        <v>-466.95076809437307</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0">
+        <v>26</v>
+      </c>
+      <c r="B28" s="0">
+        <v>-566.42470186628157</v>
+      </c>
+      <c r="C28" s="0">
+        <v>563.40570658889726</v>
+      </c>
+      <c r="D28" s="0">
+        <v>-368.75552953049339</v>
+      </c>
+      <c r="E28" s="0">
+        <v>573.13174972350419</v>
+      </c>
+      <c r="F28" s="0">
+        <v>-623.32556984134953</v>
+      </c>
+      <c r="G28" s="0">
+        <v>-471.2495518275673</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0">
+        <v>27</v>
+      </c>
+      <c r="B29" s="0">
+        <v>-572.95527253456112</v>
+      </c>
+      <c r="C29" s="0">
+        <v>573.33671985984177</v>
+      </c>
+      <c r="D29" s="0">
+        <v>-379.57175778740361</v>
+      </c>
+      <c r="E29" s="0">
+        <v>564.86386094228374</v>
+      </c>
+      <c r="F29" s="0">
+        <v>-616.1105799146693</v>
+      </c>
+      <c r="G29" s="0">
+        <v>-476.29524800952663</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0">
+        <v>28</v>
+      </c>
+      <c r="B30" s="0">
+        <v>-579.67351917819406</v>
+      </c>
+      <c r="C30" s="0">
+        <v>583.12262921492038</v>
+      </c>
+      <c r="D30" s="0">
+        <v>-390.26137863335259</v>
+      </c>
+      <c r="E30" s="0">
+        <v>556.50222073549003</v>
+      </c>
+      <c r="F30" s="0">
+        <v>-608.81535826497805</v>
+      </c>
+      <c r="G30" s="0">
+        <v>-481.97551531119598</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0">
+        <v>29</v>
+      </c>
+      <c r="B31" s="0">
+        <v>-586.57721926003285</v>
+      </c>
+      <c r="C31" s="0">
+        <v>592.76170674926277</v>
+      </c>
+      <c r="D31" s="0">
+        <v>-400.82289013066986</v>
+      </c>
+      <c r="E31" s="0">
+        <v>548.03660436168252</v>
+      </c>
+      <c r="F31" s="0">
+        <v>-601.4286347123732</v>
+      </c>
+      <c r="G31" s="0">
+        <v>-488.19551640693271</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0">
+        <v>30</v>
+      </c>
+      <c r="B32" s="0">
+        <v>-593.66412242198476</v>
+      </c>
+      <c r="C32" s="0">
+        <v>602.25205978125587</v>
+      </c>
+      <c r="D32" s="0">
+        <v>-411.25461215274078</v>
+      </c>
+      <c r="E32" s="0">
+        <v>539.45831271821317</v>
+      </c>
+      <c r="F32" s="0">
+        <v>-593.94119671645774</v>
+      </c>
+      <c r="G32" s="0">
+        <v>-494.87480120879439</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0">
+        <v>31</v>
+      </c>
+      <c r="B33" s="0">
+        <v>-600.93194766999079</v>
+      </c>
+      <c r="C33" s="0">
+        <v>611.59165542200481</v>
+      </c>
+      <c r="D33" s="0">
+        <v>-421.55471918362753</v>
+      </c>
+      <c r="E33" s="0">
+        <v>530.75994374385687</v>
+      </c>
+      <c r="F33" s="0">
+        <v>-586.34554500653712</v>
+      </c>
+      <c r="G33" s="0">
+        <v>-501.9448197822357</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0">
+        <v>32</v>
+      </c>
+      <c r="B34" s="0">
+        <v>-608.37838108256483</v>
+      </c>
+      <c r="C34" s="0">
+        <v>620.77834150740659</v>
+      </c>
+      <c r="D34" s="0">
+        <v>-431.7212677051246</v>
+      </c>
+      <c r="E34" s="0">
+        <v>521.93520278095116</v>
+      </c>
+      <c r="F34" s="0">
+        <v>-578.63561506484052</v>
+      </c>
+      <c r="G34" s="0">
+        <v>-509.34692480528997</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0">
+        <v>33</v>
+      </c>
+      <c r="B35" s="0">
+        <v>-616.00107395769624</v>
+      </c>
+      <c r="C35" s="0">
+        <v>629.80986450401883</v>
+      </c>
+      <c r="D35" s="0">
+        <v>-441.752219193222</v>
+      </c>
+      <c r="E35" s="0">
+        <v>512.97874432052595</v>
+      </c>
+      <c r="F35" s="0">
+        <v>-570.80655048776168</v>
+      </c>
+      <c r="G35" s="0">
+        <v>-517.03075753497012</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0">
+        <v>34</v>
+      </c>
+      <c r="B36" s="0">
+        <v>-623.7976413288078</v>
+      </c>
+      <c r="C36" s="0">
+        <v>638.68388488242226</v>
+      </c>
+      <c r="D36" s="0">
+        <v>-451.64545953165919</v>
+      </c>
+      <c r="E36" s="0">
+        <v>503.88603917428372</v>
+      </c>
+      <c r="F36" s="0">
+        <v>-562.85451748702053</v>
+      </c>
+      <c r="G36" s="0">
+        <v>-524.95293637901079</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0">
+        <v>35</v>
+      </c>
+      <c r="B37" s="0">
+        <v>-631.76566079304723</v>
+      </c>
+      <c r="C37" s="0">
+        <v>647.39799035913552</v>
+      </c>
+      <c r="D37" s="0">
+        <v>-461.39881548500517</v>
+      </c>
+      <c r="E37" s="0">
+        <v>494.65326235822624</v>
+      </c>
+      <c r="F37" s="0">
+        <v>-554.7765522172964</v>
+      </c>
+      <c r="G37" s="0">
+        <v>-533.07598586616473</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0">
+        <v>36</v>
+      </c>
+      <c r="B38" s="0">
+        <v>-639.90267160524991</v>
+      </c>
+      <c r="C38" s="0">
+        <v>655.94970733455762</v>
+      </c>
+      <c r="D38" s="0">
+        <v>-471.01006874531242</v>
+      </c>
+      <c r="E38" s="0">
+        <v>485.27719793027387</v>
+      </c>
+      <c r="F38" s="0">
+        <v>-546.57043444808892</v>
+      </c>
+      <c r="G38" s="0">
+        <v>-541.36745783403558</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0">
+        <v>37</v>
+      </c>
+      <c r="B39" s="0">
+        <v>-648.2061739989548</v>
+      </c>
+      <c r="C39" s="0">
+        <v>664.33651079559127</v>
+      </c>
+      <c r="D39" s="0">
+        <v>-480.47696796597262</v>
+      </c>
+      <c r="E39" s="0">
+        <v>475.75515776832504</v>
+      </c>
+      <c r="F39" s="0">
+        <v>-538.23458249133432</v>
+      </c>
+      <c r="G39" s="0">
+        <v>-549.79920726170292</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0">
+        <v>38</v>
+      </c>
+      <c r="B40" s="0">
+        <v>-656.67362870236889</v>
+      </c>
+      <c r="C40" s="0">
+        <v>672.55583290427808</v>
+      </c>
+      <c r="D40" s="0">
+        <v>-489.79723911731247</v>
+      </c>
+      <c r="E40" s="0">
+        <v>466.08491185728917</v>
+      </c>
+      <c r="F40" s="0">
+        <v>-529.7679653647856</v>
+      </c>
+      <c r="G40" s="0">
+        <v>-558.34679325943512</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0">
+        <v>39</v>
+      </c>
+      <c r="B41" s="0">
+        <v>-665.30245662244238</v>
+      </c>
+      <c r="C41" s="0">
+        <v>680.60507045552288</v>
+      </c>
+      <c r="D41" s="0">
+        <v>-498.96859443581764</v>
+      </c>
+      <c r="E41" s="0">
+        <v>456.26462811170876</v>
+      </c>
+      <c r="F41" s="0">
+        <v>-521.17002899590102</v>
+      </c>
+      <c r="G41" s="0">
+        <v>-566.98898193474315</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0">
+        <v>40</v>
+      </c>
+      <c r="B42" s="0">
+        <v>-674.09003867450974</v>
+      </c>
+      <c r="C42" s="0">
+        <v>688.48159135578385</v>
+      </c>
+      <c r="D42" s="0">
+        <v>-507.98874018892479</v>
+      </c>
+      <c r="E42" s="0">
+        <v>446.29282012336199</v>
+      </c>
+      <c r="F42" s="0">
+        <v>-512.44063391164377</v>
+      </c>
+      <c r="G42" s="0">
+        <v>-575.70733265237936</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0">
+        <v>41</v>
+      </c>
+      <c r="B43" s="0">
+        <v>-683.03371573846266</v>
+      </c>
+      <c r="C43" s="0">
+        <v>696.18274024916343</v>
+      </c>
+      <c r="D43" s="0">
+        <v>-516.85538343727865</v>
+      </c>
+      <c r="E43" s="0">
+        <v>436.16830151179863</v>
+      </c>
+      <c r="F43" s="0">
+        <v>-503.58000236020178</v>
+      </c>
+      <c r="G43" s="0">
+        <v>-584.48585293943734</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0">
+        <v>42</v>
+      </c>
+      <c r="B44" s="0">
+        <v>-692.13078872530832</v>
+      </c>
+      <c r="C44" s="0">
+        <v>703.70584339629375</v>
+      </c>
+      <c r="D44" s="0">
+        <v>-525.56623794407949</v>
+      </c>
+      <c r="E44" s="0">
+        <v>425.89014578668986</v>
+      </c>
+      <c r="F44" s="0">
+        <v>-494.58867320401635</v>
+      </c>
+      <c r="G44" s="0">
+        <v>-593.3107102107881</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0">
+        <v>43</v>
+      </c>
+      <c r="B45" s="0">
+        <v>-701.37851874033504</v>
+      </c>
+      <c r="C45" s="0">
+        <v>711.04821289409347</v>
+      </c>
+      <c r="D45" s="0">
+        <v>-534.11902935496983</v>
+      </c>
+      <c r="E45" s="0">
+        <v>415.4576508163496</v>
+      </c>
+      <c r="F45" s="0">
+        <v>-485.46746323421041</v>
+      </c>
+      <c r="G45" s="0">
+        <v>-602.16999079385721</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0">
+        <v>44</v>
+      </c>
+      <c r="B46" s="0">
+        <v>-710.77412733107474</v>
+      </c>
+      <c r="C46" s="0">
+        <v>718.20715030998531</v>
+      </c>
+      <c r="D46" s="0">
+        <v>-542.51149975058809</v>
+      </c>
+      <c r="E46" s="0">
+        <v>404.87030714639531</v>
+      </c>
+      <c r="F46" s="0">
+        <v>-476.21743380303184</v>
+      </c>
+      <c r="G46" s="0">
+        <v>-611.05349855801535</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0">
+        <v>45</v>
+      </c>
+      <c r="B47" s="0">
+        <v>-720.31479680987695</v>
+      </c>
+      <c r="C47" s="0">
+        <v>725.17994979207083</v>
+      </c>
+      <c r="D47" s="0">
+        <v>-550.74141165644255</v>
+      </c>
+      <c r="E47" s="0">
+        <v>394.12776953367495</v>
+      </c>
+      <c r="F47" s="0">
+        <v>-466.83986186741458</v>
+      </c>
+      <c r="G47" s="0">
+        <v>-619.95258691010827</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0">
+        <v>46</v>
+      </c>
+      <c r="B48" s="0">
+        <v>-729.99767064224921</v>
+      </c>
+      <c r="C48" s="0">
+        <v>731.96390070657515</v>
+      </c>
+      <c r="D48" s="0">
+        <v>-558.80655158033755</v>
+      </c>
+      <c r="E48" s="0">
+        <v>383.22983115884165</v>
+      </c>
+      <c r="F48" s="0">
+        <v>-457.33621469383911</v>
+      </c>
+      <c r="G48" s="0">
+        <v>-628.86001908561104</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0">
+        <v>47</v>
+      </c>
+      <c r="B49" s="0">
+        <v>-739.81985389324837</v>
+      </c>
+      <c r="C49" s="0">
+        <v>738.55628984522059</v>
+      </c>
+      <c r="D49" s="0">
+        <v>-566.70473313565435</v>
+      </c>
+      <c r="E49" s="0">
+        <v>372.17640006101783</v>
+      </c>
+      <c r="F49" s="0">
+        <v>-447.70812760072272</v>
+      </c>
+      <c r="G49" s="0">
+        <v>-637.76985260779804</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0">
+        <v>48</v>
+      </c>
+      <c r="B50" s="0">
+        <v>-749.77841372512501</v>
+      </c>
+      <c r="C50" s="0">
+        <v>744.95440323780974</v>
+      </c>
+      <c r="D50" s="0">
+        <v>-574.43379979880513</v>
+      </c>
+      <c r="E50" s="0">
+        <v>360.96747740304733</v>
+      </c>
+      <c r="F50" s="0">
+        <v>-437.95738421583525</v>
+      </c>
+      <c r="G50" s="0">
+        <v>-646.67734455273808</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0">
+        <v>49</v>
+      </c>
+      <c r="B51" s="0">
+        <v>-759.87037994020227</v>
+      </c>
+      <c r="C51" s="0">
+        <v>751.15552759894661</v>
+      </c>
+      <c r="D51" s="0">
+        <v>-581.99162734080721</v>
+      </c>
+      <c r="E51" s="0">
+        <v>349.60313722892119</v>
+      </c>
+      <c r="F51" s="0">
+        <v>-428.08589880771569</v>
+      </c>
+      <c r="G51" s="0">
+        <v>-655.5788748841444</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0">
+        <v>50</v>
+      </c>
+      <c r="B52" s="0">
+        <v>-770.09274556358912</v>
+      </c>
+      <c r="C52" s="0">
+        <v>757.15695143230551</v>
+      </c>
+      <c r="D52" s="0">
+        <v>-589.37612596580368</v>
+      </c>
+      <c r="E52" s="0">
+        <v>338.08350741805083</v>
+      </c>
+      <c r="F52" s="0">
+        <v>-418.09570031556132</v>
+      </c>
+      <c r="G52" s="0">
+        <v>-664.47188563767759</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0">
+        <v>51</v>
+      </c>
+      <c r="B53" s="0">
+        <v>-780.44246746085821</v>
+      </c>
+      <c r="C53" s="0">
+        <v>762.95596581101029</v>
+      </c>
+      <c r="D53" s="0">
+        <v>-596.58524218329478</v>
+      </c>
+      <c r="E53" s="0">
+        <v>326.40875157597907</v>
+      </c>
+      <c r="F53" s="0">
+        <v>-407.988917754569</v>
+      </c>
+      <c r="G53" s="0">
+        <v>-673.35483416284046</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0">
+        <v>52</v>
+      </c>
+      <c r="B54" s="0">
+        <v>-790.91646698624265</v>
+      </c>
+      <c r="C54" s="0">
+        <v>768.54986484842777</v>
+      </c>
+      <c r="D54" s="0">
+        <v>-603.61696043557981</v>
+      </c>
+      <c r="E54" s="0">
+        <v>314.57905162913932</v>
+      </c>
+      <c r="F54" s="0">
+        <v>-397.76776671553586</v>
+      </c>
+      <c r="G54" s="0">
+        <v>-682.22715898980891</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0">
+        <v>53</v>
+      </c>
+      <c r="B55" s="0">
+        <v>-801.51163065721937</v>
+      </c>
+      <c r="C55" s="0">
+        <v>773.93594586976451</v>
+      </c>
+      <c r="D55" s="0">
+        <v>-610.46930449729086</v>
+      </c>
+      <c r="E55" s="0">
+        <v>302.5945909135919</v>
+      </c>
+      <c r="F55" s="0">
+        <v>-387.43453671050486</v>
+      </c>
+      <c r="G55" s="0">
+        <v>-691.08925719330807</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0">
+        <v>54</v>
+      </c>
+      <c r="B56" s="0">
+        <v>-812.22481085163054</v>
+      </c>
+      <c r="C56" s="0">
+        <v>779.11150929142411</v>
+      </c>
+      <c r="D56" s="0">
+        <v>-617.14033865982003</v>
+      </c>
+      <c r="E56" s="0">
+        <v>290.4555375649698</v>
+      </c>
+      <c r="F56" s="0">
+        <v>-376.99157914174907</v>
+      </c>
+      <c r="G56" s="0">
+        <v>-699.94247238752075</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0">
+        <v>55</v>
+      </c>
+      <c r="B57" s="0">
+        <v>-823.05282652366736</v>
+      </c>
+      <c r="C57" s="0">
+        <v>784.07385821176194</v>
+      </c>
+      <c r="D57" s="0">
+        <v>-623.62816870970767</v>
+      </c>
+      <c r="E57" s="0">
+        <v>278.16202802996906</v>
+      </c>
+      <c r="F57" s="0">
+        <v>-366.44129569050892</v>
+      </c>
+      <c r="G57" s="0">
+        <v>-708.78909271452415</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0">
+        <v>56</v>
+      </c>
+      <c r="B58" s="0">
+        <v>-833.99246393517512</v>
+      </c>
+      <c r="C58" s="0">
+        <v>788.82029771388954</v>
+      </c>
+      <c r="D58" s="0">
+        <v>-629.93094270665597</v>
+      </c>
+      <c r="E58" s="0">
+        <v>265.71415052903444</v>
+      </c>
+      <c r="F58" s="0">
+        <v>-355.7861269354442</v>
+      </c>
+      <c r="G58" s="0">
+        <v>-717.63235839196932</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0">
+        <v>57</v>
+      </c>
+      <c r="B59" s="0">
+        <v>-845.04047739880707</v>
+      </c>
+      <c r="C59" s="0">
+        <v>793.34813387821919</v>
+      </c>
+      <c r="D59" s="0">
+        <v>-636.04685156357164</v>
+      </c>
+      <c r="E59" s="0">
+        <v>253.11192830584804</v>
+      </c>
+      <c r="F59" s="0">
+        <v>-345.02854101929069</v>
+      </c>
+      <c r="G59" s="0">
+        <v>-726.47647856994342</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="0">
+        <v>58</v>
+      </c>
+      <c r="B60" s="0">
+        <v>-856.19359002957663</v>
+      </c>
+      <c r="C60" s="0">
+        <v>797.65467249961876</v>
+      </c>
+      <c r="D60" s="0">
+        <v>-641.97412942793812</v>
+      </c>
+      <c r="E60" s="0">
+        <v>240.35530250204573</v>
+      </c>
+      <c r="F60" s="0">
+        <v>-334.17102218612837</v>
+      </c>
+      <c r="G60" s="0">
+        <v>-735.32665741822859</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="0">
+        <v>59</v>
+      </c>
+      <c r="B61" s="0">
+        <v>-867.44849450129823</v>
+      </c>
+      <c r="C61" s="0">
+        <v>801.73721750123696</v>
+      </c>
+      <c r="D61" s="0">
+        <v>-647.71105386069928</v>
+      </c>
+      <c r="E61" s="0">
+        <v>227.44411449559851</v>
+      </c>
+      <c r="F61" s="0">
+        <v>-323.21605901123275</v>
+      </c>
+      <c r="G61" s="0">
+        <v>-744.18912952823075</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="0">
+        <v>60</v>
+      </c>
+      <c r="B62" s="0">
+        <v>-878.80185380434239</v>
+      </c>
+      <c r="C62" s="0">
+        <v>805.59306903419361</v>
+      </c>
+      <c r="D62" s="0">
+        <v>-653.25594580571169</v>
+      </c>
+      <c r="E62" s="0">
+        <v>214.37808753836248</v>
+      </c>
+      <c r="F62" s="0">
+        <v>-312.16613214068963</v>
+      </c>
+      <c r="G62" s="0">
+        <v>-753.07120487337613</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0">
+        <v>61</v>
+      </c>
+      <c r="B63" s="0">
+        <v>-890.25030200095614</v>
+      </c>
+      <c r="C63" s="0">
+        <v>809.21952124944392</v>
+      </c>
+      <c r="D63" s="0">
+        <v>-658.60716933954529</v>
+      </c>
+      <c r="E63" s="0">
+        <v>201.15680752267812</v>
+      </c>
+      <c r="F63" s="0">
+        <v>-301.02370134880857</v>
+      </c>
+      <c r="G63" s="0">
+        <v>-761.98132373188196</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0">
+        <v>62</v>
+      </c>
+      <c r="B64" s="0">
+        <v>-901.79044497419977</v>
+      </c>
+      <c r="C64" s="0">
+        <v>812.61385972505946</v>
+      </c>
+      <c r="D64" s="0">
+        <v>-663.76313118795895</v>
+      </c>
+      <c r="E64" s="0">
+        <v>187.77970269845812</v>
+      </c>
+      <c r="F64" s="0">
+        <v>-289.79119170762999</v>
+      </c>
+      <c r="G64" s="0">
+        <v>-770.92912214089495</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="0">
+        <v>63</v>
+      </c>
+      <c r="B65" s="0">
+        <v>-913.41886116628928</v>
+      </c>
+      <c r="C65" s="0">
+        <v>815.77335852897693</v>
+      </c>
+      <c r="D65" s="0">
+        <v>-668.72227999162044</v>
+      </c>
+      <c r="E65" s="0">
+        <v>174.24602215068796</v>
+      </c>
+      <c r="F65" s="0">
+        <v>-278.47097864407556</v>
+      </c>
+      <c r="G65" s="0">
+        <v>-779.92550862483404</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="0">
+        <v>64</v>
+      </c>
+      <c r="B66" s="0">
+        <v>-925.13210230177833</v>
+      </c>
+      <c r="C66" s="0">
+        <v>818.69527689382062</v>
+      </c>
+      <c r="D66" s="0">
+        <v>-673.48310529953255</v>
+      </c>
+      <c r="E66" s="0">
+        <v>160.55481283277206</v>
+      </c>
+      <c r="F66" s="0">
+        <v>-267.06537163608778</v>
+      </c>
+      <c r="G66" s="0">
+        <v>-788.98275312814235</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0">
+        <v>65</v>
+      </c>
+      <c r="B67" s="0">
+        <v>-936.92669409060954</v>
+      </c>
+      <c r="C67" s="0">
+        <v>821.37685547665956</v>
+      </c>
+      <c r="D67" s="0">
+        <v>-678.04413626401742</v>
+      </c>
+      <c r="E67" s="0">
+        <v>146.70489493310572</v>
+      </c>
+      <c r="F67" s="0">
+        <v>-255.57659626863904</v>
+      </c>
+      <c r="G67" s="0">
+        <v>-798.11458928801369</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0">
+        <v>66</v>
+      </c>
+      <c r="B68" s="0">
+        <v>-948.79913690556418</v>
+      </c>
+      <c r="C68" s="0">
+        <v>823.81531217254462</v>
+      </c>
+      <c r="D68" s="0">
+        <v>-682.40394000594142</v>
+      </c>
+      <c r="E68" s="0">
+        <v>132.69483533048606</v>
+      </c>
+      <c r="F68" s="0">
+        <v>-244.00677433290258</v>
+      </c>
+      <c r="G68" s="0">
+        <v>-807.33633141132293</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0">
+        <v>67</v>
+      </c>
+      <c r="B69" s="0">
+        <v>-960.74590642803037</v>
+      </c>
+      <c r="C69" s="0">
+        <v>826.00783744611726</v>
+      </c>
+      <c r="D69" s="0">
+        <v>-686.56111961291947</v>
+      </c>
+      <c r="E69" s="0">
+        <v>118.52291886799628</v>
+      </c>
+      <c r="F69" s="0">
+        <v>-232.35790160592771</v>
+      </c>
+      <c r="G69" s="0">
+        <v>-816.66500777782915</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0">
+        <v>68</v>
+      </c>
+      <c r="B70" s="0">
+        <v>-972.76345425531986</v>
+      </c>
+      <c r="C70" s="0">
+        <v>827.95158914065564</v>
+      </c>
+      <c r="D70" s="0">
+        <v>-690.51431172647142</v>
+      </c>
+      <c r="E70" s="0">
+        <v>104.18711714412051</v>
+      </c>
+      <c r="F70" s="0">
+        <v>-220.63182289241289</v>
+      </c>
+      <c r="G70" s="0">
+        <v>-826.11951218577883</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0">
+        <v>69</v>
+      </c>
+      <c r="B71" s="0">
+        <v>-984.84820846191406</v>
+      </c>
+      <c r="C71" s="0">
+        <v>829.6436867183304</v>
+      </c>
+      <c r="D71" s="0">
+        <v>-694.26218366619753</v>
+      </c>
+      <c r="E71" s="0">
+        <v>89.685054483574817</v>
+      </c>
+      <c r="F71" s="0">
+        <v>-208.83020384273053</v>
+      </c>
+      <c r="G71" s="0">
+        <v>-835.72077599400518</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0">
+        <v>70</v>
+      </c>
+      <c r="B72" s="0">
+        <v>-996.99657410603709</v>
+      </c>
+      <c r="C72" s="0">
+        <v>831.08120487919803</v>
+      </c>
+      <c r="D72" s="0">
+        <v>-697.80343002990208</v>
+      </c>
+      <c r="E72" s="0">
+        <v>75.013970707649179</v>
+      </c>
+      <c r="F72" s="0">
+        <v>-196.95449897997645</v>
+      </c>
+      <c r="G72" s="0">
+        <v>-845.49196330652603</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0">
+        <v>71</v>
+      </c>
+      <c r="B73" s="0">
+        <v>-1009.2049336718075</v>
+      </c>
+      <c r="C73" s="0">
+        <v>832.2611664993949</v>
+      </c>
+      <c r="D73" s="0">
+        <v>-701.13676869783399</v>
+      </c>
+      <c r="E73" s="0">
+        <v>60.170680273771211</v>
+      </c>
+      <c r="F73" s="0">
+        <v>-185.00591527058143</v>
+      </c>
+      <c r="G73" s="0">
+        <v>-855.45869240229081</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0">
+        <v>72</v>
+      </c>
+      <c r="B74" s="0">
+        <v>-1021.4696474358419</v>
+      </c>
+      <c r="C74" s="0">
+        <v>833.18053482098958</v>
+      </c>
+      <c r="D74" s="0">
+        <v>-704.26093615662649</v>
+      </c>
+      <c r="E74" s="0">
+        <v>45.151527295339697</v>
+      </c>
+      <c r="F74" s="0">
+        <v>-172.98537045446639</v>
+      </c>
+      <c r="G74" s="0">
+        <v>-865.64928704861688</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0">
+        <v>73</v>
+      </c>
+      <c r="B75" s="0">
+        <v>-1033.7870537456045</v>
+      </c>
+      <c r="C75" s="0">
+        <v>833.83620481682863</v>
+      </c>
+      <c r="D75" s="0">
+        <v>-707.17468204360012</v>
+      </c>
+      <c r="E75" s="0">
+        <v>29.952335883983402</v>
+      </c>
+      <c r="F75" s="0">
+        <v>-160.89344520737171</v>
+      </c>
+      <c r="G75" s="0">
+        <v>-876.09506196795951</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0">
+        <v>74</v>
+      </c>
+      <c r="B76" s="0">
+        <v>-1046.1534691948928</v>
+      </c>
+      <c r="C76" s="0">
+        <v>834.22499364329235</v>
+      </c>
+      <c r="D76" s="0">
+        <v>-709.87676279445168</v>
+      </c>
+      <c r="E76" s="0">
+        <v>14.568355175553961</v>
+      </c>
+      <c r="F76" s="0">
+        <v>-148.73032803441657</v>
+      </c>
+      <c r="G76" s="0">
+        <v>-886.8306474750558</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0">
+        <v>75</v>
+      </c>
+      <c r="B77" s="0">
+        <v>-1058.5651886796422</v>
+      </c>
+      <c r="C77" s="0">
+        <v>834.34363008192622</v>
+      </c>
+      <c r="D77" s="0">
+        <v>-712.36593425635988</v>
+      </c>
+      <c r="E77" s="0">
+        <v>-1.0058016939008994</v>
+      </c>
+      <c r="F77" s="0">
+        <v>-136.49575158326903</v>
+      </c>
+      <c r="G77" s="0">
+        <v>-897.89435918979177</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0">
+        <v>76</v>
+      </c>
+      <c r="B78" s="0">
+        <v>-1071.0184853146193</v>
+      </c>
+      <c r="C78" s="0">
+        <v>834.18874285713105</v>
+      </c>
+      <c r="D78" s="0">
+        <v>-714.64094310347161</v>
+      </c>
+      <c r="E78" s="0">
+        <v>-16.776225508047418</v>
+      </c>
+      <c r="F78" s="0">
+        <v>-124.18891880891654</v>
+      </c>
+      <c r="G78" s="0">
+        <v>-909.328619791557</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0">
+        <v>77</v>
+      </c>
+      <c r="B79" s="0">
+        <v>-1083.5096101884451</v>
+      </c>
+      <c r="C79" s="0">
+        <v>833.75684770126247</v>
+      </c>
+      <c r="D79" s="0">
+        <v>-716.70051686174406</v>
+      </c>
+      <c r="E79" s="0">
+        <v>-32.749786764168967</v>
+      </c>
+      <c r="F79" s="0">
+        <v>-111.80841710920518</v>
+      </c>
+      <c r="G79" s="0">
+        <v>-921.18044105156036</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0">
+        <v>78</v>
+      </c>
+      <c r="B80" s="0">
+        <v>-1096.034791930759</v>
+      </c>
+      <c r="C80" s="0">
+        <v>833.04433302001985</v>
+      </c>
+      <c r="D80" s="0">
+        <v>-718.54335231404252</v>
+      </c>
+      <c r="E80" s="0">
+        <v>-48.934220475924278</v>
+      </c>
+      <c r="F80" s="0">
+        <v>-99.352118167290769</v>
+      </c>
+      <c r="G80" s="0">
+        <v>-933.50197590838252</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0">
+        <v>79</v>
+      </c>
+      <c r="B81" s="0">
+        <v>-1108.5902360609207</v>
+      </c>
+      <c r="C81" s="0">
+        <v>832.04744398968307</v>
+      </c>
+      <c r="D81" s="0">
+        <v>-720.16810201293561</v>
+      </c>
+      <c r="E81" s="0">
+        <v>-65.338221305803629</v>
+      </c>
+      <c r="F81" s="0">
+        <v>-86.817060766774972</v>
+      </c>
+      <c r="G81" s="0">
+        <v>-946.35115219859449</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="0">
+        <v>80</v>
+      </c>
+      <c r="B82" s="0">
+        <v>-1121.1721240824886</v>
+      </c>
+      <c r="C82" s="0">
+        <v>830.76226489279793</v>
+      </c>
+      <c r="D82" s="0">
+        <v>-721.57335857601913</v>
+      </c>
+      <c r="E82" s="0">
+        <v>-81.971550569743471</v>
+      </c>
+      <c r="F82" s="0">
+        <v>-74.199313265466984</v>
+      </c>
+      <c r="G82" s="0">
+        <v>-959.79240189356995</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="0">
+        <v>81</v>
+      </c>
+      <c r="B83" s="0">
+        <v>-1133.7766122814699</v>
+      </c>
+      <c r="C83" s="0">
+        <v>829.18469946974028</v>
+      </c>
+      <c r="D83" s="0">
+        <v>-722.7576363747196</v>
+      </c>
+      <c r="E83" s="0">
+        <v>-98.845156921085845</v>
+      </c>
+      <c r="F83" s="0">
+        <v>-61.493811696339392</v>
+      </c>
+      <c r="G83" s="0">
+        <v>-973.89750242037974</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="0">
+        <v>82</v>
+      </c>
+      <c r="B84" s="0">
+        <v>-1146.3998301789006</v>
+      </c>
+      <c r="C84" s="0">
+        <v>827.31044902938686</v>
+      </c>
+      <c r="D84" s="0">
+        <v>-723.71935014967607</v>
+      </c>
+      <c r="E84" s="0">
+        <v>-115.97131283852728</v>
+      </c>
+      <c r="F84" s="0">
+        <v>-48.694168573190645</v>
+      </c>
+      <c r="G84" s="0">
+        <v>-988.74654997904668</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="0">
+        <v>83</v>
+      </c>
+      <c r="B85" s="0">
+        <v>-1159.0378785793662</v>
+      </c>
+      <c r="C85" s="0">
+        <v>825.13498802178344</v>
+      </c>
+      <c r="D85" s="0">
+        <v>-724.45678999055622</v>
+      </c>
+      <c r="E85" s="0">
+        <v>-133.36376942474149</v>
+      </c>
+      <c r="F85" s="0">
+        <v>-35.792446367113676</v>
+      </c>
+      <c r="G85" s="0">
+        <v>-1004.429088863823</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="0">
+        <v>84</v>
+      </c>
+      <c r="B86" s="0">
+        <v>-1171.6868271462677</v>
+      </c>
+      <c r="C86" s="0">
+        <v>822.6535367280751</v>
+      </c>
+      <c r="D86" s="0">
+        <v>-724.96809200114001</v>
+      </c>
+      <c r="E86" s="0">
+        <v>-151.03793248391844</v>
+      </c>
+      <c r="F86" s="0">
+        <v>-22.778888227559786</v>
+      </c>
+      <c r="G86" s="0">
+        <v>-1021.0454258487783</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="0">
+        <v>85</v>
+      </c>
+      <c r="B87" s="0">
+        <v>-1184.342711421576</v>
+      </c>
+      <c r="C87" s="0">
+        <v>819.86103066640806</v>
+      </c>
+      <c r="D87" s="0">
+        <v>-725.25120382621787</v>
+      </c>
+      <c r="E87" s="0">
+        <v>-169.01106340630568</v>
+      </c>
+      <c r="F87" s="0">
+        <v>-9.6415967696411151</v>
+      </c>
+      <c r="G87" s="0">
+        <v>-1038.7081649616546</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="0">
+        <v>86</v>
+      </c>
+      <c r="B88" s="0">
+        <v>-1197.0015291919372</v>
+      </c>
+      <c r="C88" s="0">
+        <v>816.75208624519985</v>
+      </c>
+      <c r="D88" s="0">
+        <v>-725.30384403806374</v>
+      </c>
+      <c r="E88" s="0">
+        <v>-187.3025090699847</v>
+      </c>
+      <c r="F88" s="0">
+        <v>3.6338504663657742</v>
+      </c>
+      <c r="G88" s="0">
+        <v>-1057.544005772879</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="0">
+        <v>87</v>
+      </c>
+      <c r="B89" s="0">
+        <v>-1209.6592360836317</v>
+      </c>
+      <c r="C89" s="0">
+        <v>813.32096211464455</v>
+      </c>
+      <c r="D89" s="0">
+        <v>-725.12345415781931</v>
+      </c>
+      <c r="E89" s="0">
+        <v>-205.93396580480297</v>
+      </c>
+      <c r="F89" s="0">
+        <v>17.064863093213308</v>
+      </c>
+      <c r="G89" s="0">
+        <v>-1077.6958580977794</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="0">
+        <v>88</v>
+      </c>
+      <c r="B90" s="0">
+        <v>-1222.3117402451835</v>
+      </c>
+      <c r="C90" s="0">
+        <v>809.56151557062503</v>
+      </c>
+      <c r="D90" s="0">
+        <v>-724.70714180899108</v>
+      </c>
+      <c r="E90" s="0">
+        <v>-224.92978348986824</v>
+      </c>
+      <c r="F90" s="0">
+        <v>30.672395300259172</v>
+      </c>
+      <c r="G90" s="0">
+        <v>-1099.3253383121582</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="0">
+        <v>89</v>
+      </c>
+      <c r="B91" s="0">
+        <v>-1234.9548959472431</v>
+      </c>
+      <c r="C91" s="0">
+        <v>805.46715324857348</v>
+      </c>
+      <c r="D91" s="0">
+        <v>-724.05161315084695</v>
+      </c>
+      <c r="E91" s="0">
+        <v>-244.31731712446413</v>
+      </c>
+      <c r="F91" s="0">
+        <v>44.481621052435713</v>
+      </c>
+      <c r="G91" s="0">
+        <v>-1122.6157280586906</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="0">
+        <v>90</v>
+      </c>
+      <c r="B92" s="0">
+        <v>-1247.5844958933558</v>
+      </c>
+      <c r="C92" s="0">
+        <v>801.03077520344709</v>
+      </c>
+      <c r="D92" s="0">
+        <v>-723.15309229812056</v>
+      </c>
+      <c r="E92" s="0">
+        <v>-264.12733478819257</v>
+      </c>
+      <c r="F92" s="0">
+        <v>58.522755468392027</v>
+      </c>
+      <c r="G92" s="0">
+        <v>-1147.775495964064</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="0">
+        <v>91</v>
+      </c>
+      <c r="B93" s="0">
+        <v>-1260.1962619904862</v>
+      </c>
+      <c r="C93" s="0">
+        <v>796.24471129986762</v>
+      </c>
+      <c r="D93" s="0">
+        <v>-722.00722487292535</v>
+      </c>
+      <c r="E93" s="0">
+        <v>-284.39449287493983</v>
+      </c>
+      <c r="F93" s="0">
+        <v>72.832058549619731</v>
+      </c>
+      <c r="G93" s="0">
+        <v>-1175.0425084226852</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="0">
+        <v>92</v>
+      </c>
+      <c r="B94" s="0">
+        <v>-1272.7858342723855</v>
+      </c>
+      <c r="C94" s="0">
+        <v>791.10064862570812</v>
+      </c>
+      <c r="D94" s="0">
+        <v>-720.60896211872887</v>
+      </c>
+      <c r="E94" s="0">
+        <v>-305.15789195954392</v>
+      </c>
+      <c r="F94" s="0">
+        <v>87.453067599955546</v>
+      </c>
+      <c r="G94" s="0">
+        <v>-1204.6890883262147</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="0">
+        <v>93</v>
+      </c>
+      <c r="B95" s="0">
+        <v>-1285.3487575988561</v>
+      </c>
+      <c r="C95" s="0">
+        <v>785.58954838307022</v>
+      </c>
+      <c r="D95" s="0">
+        <v>-718.95242108599905</v>
+      </c>
+      <c r="E95" s="0">
+        <v>-326.46172978468928</v>
+      </c>
+      <c r="F95" s="0">
+        <v>102.43811807522525</v>
+      </c>
+      <c r="G95" s="0">
+        <v>-1237.0281232740858</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="0">
+        <v>94</v>
+      </c>
+      <c r="B96" s="0">
+        <v>-1297.8804656656948</v>
+      </c>
+      <c r="C96" s="0">
+        <v>779.70155038945154</v>
+      </c>
+      <c r="D96" s="0">
+        <v>-717.03071520860942</v>
+      </c>
+      <c r="E96" s="0">
+        <v>-348.35607183831297</v>
+      </c>
+      <c r="F96" s="0">
+        <v>117.85023039361633</v>
+      </c>
+      <c r="G96" s="0">
+        <v>-1272.4204806484126</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0">
+        <v>95</v>
+      </c>
+      <c r="B97" s="0">
+        <v>-1310.3762617479829</v>
+      </c>
+      <c r="C97" s="0">
+        <v>773.42586292198973</v>
+      </c>
+      <c r="D97" s="0">
+        <v>-714.83574803942872</v>
+      </c>
+      <c r="E97" s="0">
+        <v>-370.89776509695974</v>
+      </c>
+      <c r="F97" s="0">
+        <v>133.76546404083848</v>
+      </c>
+      <c r="G97" s="0">
+        <v>-1311.284060637408</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="0">
+        <v>96</v>
+      </c>
+      <c r="B98" s="0">
+        <v>-1322.8312954562568</v>
+      </c>
+      <c r="C98" s="0">
+        <v>766.75063513620921</v>
+      </c>
+      <c r="D98" s="0">
+        <v>-712.35796087881249</v>
+      </c>
+      <c r="E98" s="0">
+        <v>-394.15152710364362</v>
+      </c>
+      <c r="F98" s="0">
+        <v>150.2758724160314</v>
+      </c>
+      <c r="G98" s="0">
+        <v>-1354.1049163712266</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="0">
+        <v>97</v>
+      </c>
+      <c r="B99" s="0">
+        <v>-1335.2405346009828</v>
+      </c>
+      <c r="C99" s="0">
+        <v>759.66280865769841</v>
+      </c>
+      <c r="D99" s="0">
+        <v>-709.5860223391237</v>
+      </c>
+      <c r="E99" s="0">
+        <v>-418.19125113118758</v>
+      </c>
+      <c r="F99" s="0">
+        <v>167.49323556647082</v>
+      </c>
+      <c r="G99" s="0">
+        <v>-1401.4510020296802</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="0">
+        <v>98</v>
+      </c>
+      <c r="B100" s="0">
+        <v>-1347.5987310222849</v>
+      </c>
+      <c r="C100" s="0">
+        <v>752.14794414014182</v>
+      </c>
+      <c r="D100" s="0">
+        <v>-706.50644430076602</v>
+      </c>
+      <c r="E100" s="0">
+        <v>-443.10157944854655</v>
+      </c>
+      <c r="F100" s="0">
+        <v>185.55380799400743</v>
+      </c>
+      <c r="G100" s="0">
+        <v>-1453.9892883066568</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="0">
+        <v>99</v>
+      </c>
+      <c r="B101" s="0">
+        <v>-1359.9003789305746</v>
+      </c>
+      <c r="C101" s="0">
+        <v>744.19001755115994</v>
+      </c>
+      <c r="D101" s="0">
+        <v>-703.10310388888172</v>
+      </c>
+      <c r="E101" s="0">
+        <v>-468.97981163256571</v>
+      </c>
+      <c r="F101" s="0">
+        <v>204.62440201787075</v>
+      </c>
+      <c r="G101" s="0">
+        <v>-1512.5072291045356</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="0">
+        <v>100</v>
+      </c>
+      <c r="B102" s="0">
+        <v>-1372.1396638939371</v>
+      </c>
+      <c r="C102" s="0">
+        <v>735.77117961342481</v>
+      </c>
+      <c r="D102" s="0">
+        <v>-699.35664454506525</v>
+      </c>
+      <c r="E102" s="0">
+        <v>-495.93823483072265</v>
+      </c>
+      <c r="F102" s="0">
+        <v>224.91024401047511</v>
+      </c>
+      <c r="G102" s="0">
+        <v>-1577.9399018295935</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="0">
+        <v>101</v>
+      </c>
+      <c r="B103" s="0">
+        <v>-1384.3104000639139</v>
+      </c>
+      <c r="C103" s="0">
+        <v>726.87147008831221</v>
+      </c>
+      <c r="D103" s="0">
+        <v>-695.24372027489665</v>
+      </c>
+      <c r="E103" s="0">
+        <v>-524.1069898620849</v>
+      </c>
+      <c r="F103" s="0">
+        <v>246.66520658131441</v>
+      </c>
+      <c r="G103" s="0">
+        <v>-1651.4046178441934</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="0">
+        <v>102</v>
+      </c>
+      <c r="B104" s="0">
+        <v>-1396.4059525015573</v>
+      </c>
+      <c r="C104" s="0">
+        <v>717.46847629679871</v>
+      </c>
+      <c r="D104" s="0">
+        <v>-690.73603467582006</v>
+      </c>
+      <c r="E104" s="0">
+        <v>-553.63762392233457</v>
+      </c>
+      <c r="F104" s="0">
+        <v>270.20525789636406</v>
+      </c>
+      <c r="G104" s="0">
+        <v>-1734.2454723328724</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="0">
+        <v>103</v>
+      </c>
+      <c r="B105" s="0">
+        <v>-1408.4191404769135</v>
+      </c>
+      <c r="C105" s="0">
+        <v>707.53692222026382</v>
+      </c>
+      <c r="D105" s="0">
+        <v>-685.79910883553328</v>
+      </c>
+      <c r="E105" s="0">
+        <v>-584.70753167798114</v>
+      </c>
+      <c r="F105" s="0">
+        <v>295.92631598784004</v>
+      </c>
+      <c r="G105" s="0">
+        <v>-1828.0912702670093</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="0">
+        <v>104</v>
+      </c>
+      <c r="B106" s="0">
+        <v>-1420.3421162603668</v>
+      </c>
+      <c r="C106" s="0">
+        <v>697.04817041371644</v>
+      </c>
+      <c r="D106" s="0">
+        <v>-680.39068728539564</v>
+      </c>
+      <c r="E106" s="0">
+        <v>-617.5255580483007</v>
+      </c>
+      <c r="F106" s="0">
+        <v>324.32820801254104</v>
+      </c>
+      <c r="G106" s="0">
+        <v>-1934.9316771295189</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="0">
+        <v>105</v>
+      </c>
+      <c r="B107" s="0">
+        <v>-1432.1662120452661</v>
+      </c>
+      <c r="C107" s="0">
+        <v>685.96961335963772</v>
+      </c>
+      <c r="D107" s="0">
+        <v>-674.45865527812544</v>
+      </c>
+      <c r="E107" s="0">
+        <v>-652.33913765158172</v>
+      </c>
+      <c r="F107" s="0">
+        <v>356.04720295789804</v>
+      </c>
+      <c r="G107" s="0">
+        <v>-2057.2185372007152</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="0">
+        <v>106</v>
+      </c>
+      <c r="B108" s="0">
+        <v>-1443.8817450001698</v>
+      </c>
+      <c r="C108" s="0">
+        <v>674.26392314480427</v>
+      </c>
+      <c r="D108" s="0">
+        <v>-667.93828807018713</v>
+      </c>
+      <c r="E108" s="0">
+        <v>-689.44349272176578</v>
+      </c>
+      <c r="F108" s="0">
+        <v>391.90075975504868</v>
+      </c>
+      <c r="G108" s="0">
+        <v>-2198.0024629071299</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="0">
+        <v>107</v>
+      </c>
+      <c r="B109" s="0">
+        <v>-1455.4777666821574</v>
+      </c>
+      <c r="C109" s="0">
+        <v>661.88811747604495</v>
+      </c>
+      <c r="D109" s="0">
+        <v>-660.74857458645261</v>
+      </c>
+      <c r="E109" s="0">
+        <v>-729.19362697109921</v>
+      </c>
+      <c r="F109" s="0">
+        <v>432.94995866971743</v>
+      </c>
+      <c r="G109" s="0">
+        <v>-2361.1196614871842</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="0">
+        <v>108</v>
+      </c>
+      <c r="B110" s="0">
+        <v>-1466.9417375833068</v>
+      </c>
+      <c r="C110" s="0">
+        <v>648.79238455609971</v>
+      </c>
+      <c r="D110" s="0">
+        <v>-652.78723908778739</v>
+      </c>
+      <c r="E110" s="0">
+        <v>-772.02017563994957</v>
+      </c>
+      <c r="F110" s="0">
+        <v>480.58798470118012</v>
+      </c>
+      <c r="G110" s="0">
+        <v>-2551.4516058814106</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="0">
+        <v>109</v>
+      </c>
+      <c r="B111" s="0">
+        <v>-1478.2590995284281</v>
+      </c>
+      <c r="C111" s="0">
+        <v>634.91858684325393</v>
+      </c>
+      <c r="D111" s="0">
+        <v>-643.92390064508777</v>
+      </c>
+      <c r="E111" s="0">
+        <v>-818.45066510596189</v>
+      </c>
+      <c r="F111" s="0">
+        <v>536.66774764954209</v>
+      </c>
+      <c r="G111" s="0">
+        <v>-2775.2924449701304</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="0">
+        <v>110</v>
+      </c>
+      <c r="B112" s="0">
+        <v>-1489.4127065237672</v>
+      </c>
+      <c r="C112" s="0">
+        <v>620.1983303916968</v>
+      </c>
+      <c r="D112" s="0">
+        <v>-633.99051918708392</v>
+      </c>
+      <c r="E112" s="0">
+        <v>-869.13850634114965</v>
+      </c>
+      <c r="F112" s="0">
+        <v>603.68958891249338</v>
+      </c>
+      <c r="G112" s="0">
+        <v>-3040.8793287389653</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="0">
+        <v>111</v>
+      </c>
+      <c r="B113" s="0">
+        <v>-1500.3820560159775</v>
+      </c>
+      <c r="C113" s="0">
+        <v>604.55043598253178</v>
+      </c>
+      <c r="D113" s="0">
+        <v>-622.76780427416827</v>
+      </c>
+      <c r="E113" s="0">
+        <v>-924.90328299930866</v>
+      </c>
+      <c r="F113" s="0">
+        <v>685.08352424522752</v>
+      </c>
+      <c r="G113" s="0">
+        <v>-3359.1752762237693</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="0">
+        <v>112</v>
+      </c>
+      <c r="B114" s="0">
+        <v>-1511.1422331273982</v>
+      </c>
+      <c r="C114" s="0">
+        <v>587.87756981955397</v>
+      </c>
+      <c r="D114" s="0">
+        <v>-609.96547306312755</v>
+      </c>
+      <c r="E114" s="0">
+        <v>-986.7879362161201</v>
+      </c>
+      <c r="F114" s="0">
+        <v>785.64439928518323</v>
+      </c>
+      <c r="G114" s="0">
+        <v>-3745.0546758697829</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="0">
+        <v>113</v>
+      </c>
+      <c r="B115" s="0">
+        <v>-1521.6624327608333</v>
+      </c>
+      <c r="C115" s="0">
+        <v>570.06166617854672</v>
+      </c>
+      <c r="D115" s="0">
+        <v>-595.1928810410592</v>
+      </c>
+      <c r="E115" s="0">
+        <v>-1056.1419301638111</v>
+      </c>
+      <c r="F115" s="0">
+        <v>912.22232829199118</v>
+      </c>
+      <c r="G115" s="0">
+        <v>-4219.1516010303303</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="0">
+        <v>114</v>
+      </c>
+      <c r="B116" s="0">
+        <v>-1531.9038446143791</v>
+      </c>
+      <c r="C116" s="0">
+        <v>550.95756731222491</v>
+      </c>
+      <c r="D116" s="0">
+        <v>-577.91410815961456</v>
+      </c>
+      <c r="E116" s="0">
+        <v>-1134.7456480659116</v>
+      </c>
+      <c r="F116" s="0">
+        <v>1074.8551387075333</v>
+      </c>
+      <c r="G116" s="0">
+        <v>-4810.8402292784567</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="0">
+        <v>115</v>
+      </c>
+      <c r="B117" s="0">
+        <v>-1541.8165473161521</v>
+      </c>
+      <c r="C117" s="0">
+        <v>530.38395076101494</v>
+      </c>
+      <c r="D117" s="0">
+        <v>-557.37701975514028</v>
+      </c>
+      <c r="E117" s="0">
+        <v>-1225.0026681393749</v>
+      </c>
+      <c r="F117" s="0">
+        <v>1288.6993253624612</v>
+      </c>
+      <c r="G117" s="0">
+        <v>-5563.2336837526891</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="0">
+        <v>116</v>
+      </c>
+      <c r="B118" s="0">
+        <v>-1551.3348057701871</v>
+      </c>
+      <c r="C118" s="0">
+        <v>508.10997774537503</v>
+      </c>
+      <c r="D118" s="0">
+        <v>-532.49685173403827</v>
+      </c>
+      <c r="E118" s="0">
+        <v>-1330.2487380483935</v>
+      </c>
+      <c r="F118" s="0">
+        <v>1577.4777633955469</v>
+      </c>
+      <c r="G118" s="0">
+        <v>-6541.9682288206759</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="0">
+        <v>117</v>
+      </c>
+      <c r="B119" s="0">
+        <v>-1560.3696836618913</v>
+      </c>
+      <c r="C119" s="0">
+        <v>483.8348946642036</v>
+      </c>
+      <c r="D119" s="0">
+        <v>-501.65615396413358</v>
+      </c>
+      <c r="E119" s="0">
+        <v>-1455.2720417015626</v>
+      </c>
+      <c r="F119" s="0">
+        <v>1979.9872028835494</v>
+      </c>
+      <c r="G119" s="0">
+        <v>-7851.5300150036346</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="0">
+        <v>118</v>
+      </c>
+      <c r="B120" s="0">
+        <v>-1568.7969016599866</v>
+      </c>
+      <c r="C120" s="0">
+        <v>457.15540397809332</v>
+      </c>
+      <c r="D120" s="0">
+        <v>-462.34095472707867</v>
+      </c>
+      <c r="E120" s="0">
+        <v>-1607.2409681845643</v>
+      </c>
+      <c r="F120" s="0">
+        <v>2563.2500227624041</v>
+      </c>
+      <c r="G120" s="0">
+        <v>-9667.7656018533762</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="0">
+        <v>119</v>
+      </c>
+      <c r="B121" s="0">
+        <v>-1576.4357142519343</v>
+      </c>
+      <c r="C121" s="0">
+        <v>427.51037359978557</v>
+      </c>
+      <c r="D121" s="0">
+        <v>-410.43009369720574</v>
+      </c>
+      <c r="E121" s="0">
+        <v>-1797.4822928477629</v>
+      </c>
+      <c r="F121" s="0">
+        <v>3451.4903123511158</v>
+      </c>
+      <c r="G121" s="0">
+        <v>-12308.491306037176</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="0">
+        <v>120</v>
+      </c>
+      <c r="B122" s="0">
+        <v>-1583.0093475396702</v>
+      </c>
+      <c r="C122" s="0">
+        <v>394.07988244736203</v>
+      </c>
+      <c r="D122" s="0">
+        <v>-338.67187070637317</v>
+      </c>
+      <c r="E122" s="0">
+        <v>-2045.2239665465415</v>
+      </c>
+      <c r="F122" s="0">
+        <v>4897.5944653579854</v>
+      </c>
+      <c r="G122" s="0">
+        <v>-16405.233110993599</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>